<commit_message>
feat: oto-ikmal (sonsuz içerik) — infinite-trip yeniden aktif (Part 11-15)
Gemini yönetmen stok azalınca yeni bölüm planlarını kendisi yazar
(series/replenish.py, opt-in auto_replenish). infinite-trip: bölüm içi
zincir (chain_scope=episode) + micro_trim + hook_teaser açıldı; Part 11
'Celestial Ribbons' yerelde üretildi, 3 platformda yayında (next_part=12).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/series_data/infinite-trip/series_log.xlsx
+++ b/series_data/infinite-trip/series_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2797,6 +2797,226 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>105.0</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/082cd547b430a8704bd790bfd8318f77_1783022570.mp4</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\infinite-trip\episodes\ep11\shots\shot_01.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>105.0</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/d9ef0b8bc010585ff040478c8da77baa_1783022848.mp4</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\infinite-trip\episodes\ep11\shots\shot_02.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>105.0</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/41f0769826ab2bd19f17a47985dfa740_1783023120.mp4</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\infinite-trip\episodes\ep11\shots\shot_03.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>1080p</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>105.0</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://tempfile.aiquickdraw.com/v/f8f1f51ea19eb452a72ab621fbe8caa6_1783023248.mp4</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>C:\Users\ihsan\Desktop\Antigravity\Projects\Youtube\output\series\infinite-trip\episodes\ep11\shots\shot_04.mp4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>